<commit_message>
added todolist, currently there are still probelems with reading in the xlsx file with the vocabulary.
</commit_message>
<xml_diff>
--- a/VOCABS.xlsx
+++ b/VOCABS.xlsx
@@ -1865,28 +1865,28 @@
     <t xml:space="preserve">Leder</t>
   </si>
   <si>
+    <t xml:space="preserve">snoek</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hecht</t>
   </si>
   <si>
-    <t xml:space="preserve">snoek</t>
+    <t xml:space="preserve">snoekbars</t>
   </si>
   <si>
     <t xml:space="preserve">Zander</t>
   </si>
   <si>
-    <t xml:space="preserve">snoekbaars</t>
+    <t xml:space="preserve">ontsteking</t>
   </si>
   <si>
     <t xml:space="preserve">Entzündung</t>
   </si>
   <si>
-    <t xml:space="preserve">ontsteking</t>
+    <t xml:space="preserve">volop</t>
   </si>
   <si>
     <t xml:space="preserve">vollständig</t>
-  </si>
-  <si>
-    <t xml:space="preserve">volop</t>
   </si>
   <si>
     <t xml:space="preserve">plakband</t>

</xml_diff>